<commit_message>
﻿Mise à jour ADMINISTRATEUR DE VENTE : données Janvier → Septembre (2025 vs 2026)
- Nouveau script update_admin_vente_janv_sept.py : méthodologie v2 conservée (cat_map pour
  les deux années, Montant HT, état Livrée ; services Validée côté 2026), étendue à Jan-Sep
- 2026 : S1 + ERP juillet (9), août (27), septembre (51)
- 2025 : fichier 86d96135 étendu à septembre (volume M1051 recalculé qté×50kg)
- Correction cat_map : MAT015, MAT011-80010002, MAT014-80010003 → ALVEOLE
  (alvéoles gros/petit trou classées à tort en DIVERS côté 2025)
- Fichier rempli conservé : valeurs remplacées, structure et formules intactes (PREMIX R51, Total)
- admin_vente_data_janv_sept.json + premix_ca.json (Jan-Sep) archivés

Co-Authored-By: Claude Code <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/download/ADMINISTRATEUR_DE_VENTE_rempli.xlsx
+++ b/download/ADMINISTRATEUR_DE_VENTE_rempli.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CAHT par agence A" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ventes par produits A" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vente en volume A" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="CAHT par agence A" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Ventes par produits A" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Vente en volume A" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -3207,14 +3207,14 @@
         </is>
       </c>
       <c r="B117" s="9" t="n">
-        <v>1761622350.53</v>
+        <v>2880085443.32</v>
       </c>
       <c r="C117" s="10">
         <f>+B117/$B$95</f>
         <v/>
       </c>
       <c r="D117" s="9" t="n">
-        <v>1344326244</v>
+        <v>2041232489</v>
       </c>
       <c r="E117" s="10">
         <f>+D117/D131</f>
@@ -3241,14 +3241,14 @@
         </is>
       </c>
       <c r="B118" s="9" t="n">
-        <v>967768360.4400001</v>
+        <v>1641753982.31</v>
       </c>
       <c r="C118" s="10">
         <f>+B118/$B$95</f>
         <v/>
       </c>
       <c r="D118" s="9" t="n">
-        <v>745337251</v>
+        <v>1181614830</v>
       </c>
       <c r="E118" s="10">
         <f>+D118/D131</f>
@@ -3275,14 +3275,14 @@
         </is>
       </c>
       <c r="B119" s="9" t="n">
-        <v>558163316.67</v>
+        <v>991959784.54</v>
       </c>
       <c r="C119" s="10">
         <f>+B119/$B$95</f>
         <v/>
       </c>
       <c r="D119" s="9" t="n">
-        <v>399886115</v>
+        <v>679683768</v>
       </c>
       <c r="E119" s="10">
         <f>+D119/D131</f>
@@ -3309,14 +3309,14 @@
         </is>
       </c>
       <c r="B120" s="9" t="n">
-        <v>359991116</v>
+        <v>577728822.12</v>
       </c>
       <c r="C120" s="10">
         <f>+B120/$B$95</f>
         <v/>
       </c>
       <c r="D120" s="9" t="n">
-        <v>216719901</v>
+        <v>366105542</v>
       </c>
       <c r="E120" s="10">
         <f>+D120/D131</f>
@@ -3343,14 +3343,14 @@
         </is>
       </c>
       <c r="B121" s="9" t="n">
-        <v>833521499</v>
+        <v>1417766654.55</v>
       </c>
       <c r="C121" s="10">
         <f>+B121/$B$95</f>
         <v/>
       </c>
       <c r="D121" s="9" t="n">
-        <v>797491248</v>
+        <v>1202508955</v>
       </c>
       <c r="E121" s="10">
         <f>+D121/D131</f>
@@ -3377,14 +3377,14 @@
         </is>
       </c>
       <c r="B122" s="9" t="n">
-        <v>557708133</v>
+        <v>876206317.53</v>
       </c>
       <c r="C122" s="10">
         <f>+B122/$B$95</f>
         <v/>
       </c>
       <c r="D122" s="9" t="n">
-        <v>369421977</v>
+        <v>589782613</v>
       </c>
       <c r="E122" s="10">
         <f>+D122/D131</f>
@@ -3411,14 +3411,14 @@
         </is>
       </c>
       <c r="B123" s="9" t="n">
-        <v>4451042325</v>
+        <v>7241314659.62</v>
       </c>
       <c r="C123" s="10">
         <f>+B123/$B$95</f>
         <v/>
       </c>
       <c r="D123" s="9" t="n">
-        <v>4740291755</v>
+        <v>6649942780</v>
       </c>
       <c r="E123" s="10">
         <f>+D123/D131</f>
@@ -3445,14 +3445,14 @@
         </is>
       </c>
       <c r="B124" s="9" t="n">
-        <v>1343143247.45</v>
+        <v>2451046150.95</v>
       </c>
       <c r="C124" s="10">
         <f>+B124/$B$95</f>
         <v/>
       </c>
       <c r="D124" s="9" t="n">
-        <v>1019774150</v>
+        <v>1499410596</v>
       </c>
       <c r="E124" s="10">
         <f>+D124/D131</f>
@@ -3479,14 +3479,14 @@
         </is>
       </c>
       <c r="B125" s="9" t="n">
-        <v>1028147860</v>
+        <v>1716103866.29</v>
       </c>
       <c r="C125" s="10">
         <f>+B125/$B$95</f>
         <v/>
       </c>
       <c r="D125" s="9" t="n">
-        <v>719127200</v>
+        <v>1035764760</v>
       </c>
       <c r="E125" s="10">
         <f>+D125/D131</f>
@@ -3513,14 +3513,14 @@
         </is>
       </c>
       <c r="B126" s="9" t="n">
-        <v>710749845</v>
+        <v>1097141014.61</v>
       </c>
       <c r="C126" s="10">
         <f>+B126/$B$95</f>
         <v/>
       </c>
       <c r="D126" s="9" t="n">
-        <v>698497782</v>
+        <v>1042583624</v>
       </c>
       <c r="E126" s="10">
         <f>+D126/D131</f>
@@ -3547,14 +3547,14 @@
         </is>
       </c>
       <c r="B127" s="9" t="n">
-        <v>589719790.59</v>
+        <v>915735275.1799999</v>
       </c>
       <c r="C127" s="10">
         <f>+B127/$B$95</f>
         <v/>
       </c>
       <c r="D127" s="9" t="n">
-        <v>628656257</v>
+        <v>921048169</v>
       </c>
       <c r="E127" s="10">
         <f>+D127/D131</f>
@@ -3581,14 +3581,14 @@
         </is>
       </c>
       <c r="B128" s="9" t="n">
-        <v>948464421.04</v>
+        <v>1508982191.58</v>
       </c>
       <c r="C128" s="10">
         <f>+B128/$B$95</f>
         <v/>
       </c>
       <c r="D128" s="9" t="n">
-        <v>756796677</v>
+        <v>1153123492</v>
       </c>
       <c r="E128" s="10">
         <f>+D128/D131</f>
@@ -3615,14 +3615,14 @@
         </is>
       </c>
       <c r="B129" s="9" t="n">
-        <v>2565427193.29</v>
+        <v>3986108240.15</v>
       </c>
       <c r="C129" s="10">
         <f>+B129/$B$95</f>
         <v/>
       </c>
       <c r="D129" s="9" t="n">
-        <v>3152050715</v>
+        <v>4091814437</v>
       </c>
       <c r="E129" s="10">
         <f>+D129/D131</f>
@@ -3649,14 +3649,14 @@
         </is>
       </c>
       <c r="B130" s="9" t="n">
-        <v>637266987.72</v>
+        <v>1105640695.52</v>
       </c>
       <c r="C130" s="10">
         <f>+B130/$B$95</f>
         <v/>
       </c>
       <c r="D130" s="9" t="n">
-        <v>479332323</v>
+        <v>730538340</v>
       </c>
       <c r="E130" s="10">
         <f>+D130/D131</f>
@@ -5113,14 +5113,14 @@
         </is>
       </c>
       <c r="L46" s="19" t="n">
-        <v>9437426044</v>
+        <v>16129702855</v>
       </c>
       <c r="M46" s="14">
         <f>+L46/L$56</f>
         <v/>
       </c>
       <c r="N46" s="19" t="n">
-        <v>7513857160</v>
+        <v>10604533532</v>
       </c>
       <c r="O46" s="14">
         <f>+N46/N$56</f>
@@ -5142,14 +5142,14 @@
         </is>
       </c>
       <c r="L47" s="19" t="n">
-        <v>644794632.73</v>
+        <v>1009707674.27</v>
       </c>
       <c r="M47" s="14">
         <f>+L47/L$56</f>
         <v/>
       </c>
       <c r="N47" s="19" t="n">
-        <v>635908389</v>
+        <v>1065677989</v>
       </c>
       <c r="O47" s="14">
         <f>+N47/N$56</f>
@@ -5171,14 +5171,14 @@
         </is>
       </c>
       <c r="L48" s="19" t="n">
-        <v>128803200</v>
+        <v>245193950</v>
       </c>
       <c r="M48" s="14">
         <f>+L48/L$56</f>
         <v/>
       </c>
       <c r="N48" s="19" t="n">
-        <v>65993800</v>
+        <v>122803550</v>
       </c>
       <c r="O48" s="14">
         <f>+N48/N$56</f>
@@ -5200,14 +5200,14 @@
         </is>
       </c>
       <c r="L49" s="19" t="n">
-        <v>470569816</v>
+        <v>744218759</v>
       </c>
       <c r="M49" s="14">
         <f>+L49/L$56</f>
         <v/>
       </c>
       <c r="N49" s="19" t="n">
-        <v>310441909</v>
+        <v>486127901</v>
       </c>
       <c r="O49" s="14">
         <f>+N49/N$56</f>
@@ -5229,14 +5229,14 @@
         </is>
       </c>
       <c r="L50" s="19" t="n">
-        <v>6064377053</v>
+        <v>9685233807</v>
       </c>
       <c r="M50" s="14">
         <f>+L50/L$56</f>
         <v/>
       </c>
       <c r="N50" s="19" t="n">
-        <v>6113507625</v>
+        <v>9113080068</v>
       </c>
       <c r="O50" s="14">
         <f>+N50/N$56</f>
@@ -5258,14 +5258,14 @@
         </is>
       </c>
       <c r="L51" t="n">
-        <v>126044000</v>
+        <v>175347000</v>
       </c>
       <c r="M51">
         <f>+L51/L$56</f>
         <v/>
       </c>
       <c r="N51" t="n">
-        <v>87950400</v>
+        <v>133281400</v>
       </c>
       <c r="O51">
         <f>+N51/N$56</f>
@@ -5287,14 +5287,14 @@
         </is>
       </c>
       <c r="L52" s="19" t="n">
-        <v>19328750</v>
+        <v>28494550</v>
       </c>
       <c r="M52" s="14">
         <f>+L52/L$56</f>
         <v/>
       </c>
       <c r="N52" s="19" t="n">
-        <v>386499722</v>
+        <v>52951865</v>
       </c>
       <c r="O52" s="14">
         <f>+N52/N$56</f>
@@ -5316,14 +5316,14 @@
         </is>
       </c>
       <c r="L53" s="19" t="n">
-        <v>12915750</v>
+        <v>16686803</v>
       </c>
       <c r="M53" s="14">
         <f>+L53/L$56</f>
         <v/>
       </c>
       <c r="N53" s="19" t="n">
-        <v>14145960</v>
+        <v>20633160</v>
       </c>
       <c r="O53" s="14">
         <f>+N53/N$56</f>
@@ -5345,14 +5345,14 @@
         </is>
       </c>
       <c r="L54" s="19" t="n">
-        <v>13778500</v>
+        <v>27752950</v>
       </c>
       <c r="M54" s="14">
         <f>+L54/L$56</f>
         <v/>
       </c>
       <c r="N54" s="19" t="n">
-        <v>19293450</v>
+        <v>851559250</v>
       </c>
       <c r="O54" s="14">
         <f>+N54/N$56</f>
@@ -5871,10 +5871,10 @@
         </is>
       </c>
       <c r="D24" s="26" t="n">
-        <v>29061.47</v>
+        <v>45621.88</v>
       </c>
       <c r="E24" s="25" t="n">
-        <v>20794.27</v>
+        <v>30131.35</v>
       </c>
       <c r="F24" s="34">
         <f>+D24-E24</f>
@@ -5893,10 +5893,10 @@
         </is>
       </c>
       <c r="D25" s="26" t="n">
-        <v>489.99</v>
+        <v>742.9299999999999</v>
       </c>
       <c r="E25" s="25" t="n">
-        <v>499.57</v>
+        <v>797.4299999999999</v>
       </c>
       <c r="F25" s="34">
         <f>+D25-E25</f>
@@ -5937,10 +5937,10 @@
         </is>
       </c>
       <c r="D27" s="26" t="n">
-        <v>545.16</v>
+        <v>859.61</v>
       </c>
       <c r="E27" s="25" t="n">
-        <v>360.45</v>
+        <v>561.72</v>
       </c>
       <c r="F27" s="34">
         <f>+D27-E27</f>
@@ -5959,10 +5959,10 @@
         </is>
       </c>
       <c r="D28" s="26" t="n">
-        <v>9075.4</v>
+        <v>14454.07</v>
       </c>
       <c r="E28" s="25" t="n">
-        <v>9251.200000000001</v>
+        <v>13787.11</v>
       </c>
       <c r="F28" s="34">
         <f>+D28-E28</f>
@@ -5981,10 +5981,10 @@
         </is>
       </c>
       <c r="D29" s="26" t="n">
-        <v>5.06</v>
+        <v>7.51</v>
       </c>
       <c r="E29" s="25" t="n">
-        <v>19.06</v>
+        <v>21.92</v>
       </c>
       <c r="F29" s="34">
         <f>+D29-E29</f>

</xml_diff>

<commit_message>
ADMINISTRATEUR DE VENTE : données Janvier → Octobre (2025 vs 2026), arrêtées au 05/10
- Septembre basculé sur le bilan définitif (61), octobre MTD ajouté (60, 01-05/10)
- 2025 tronqué au 05/10 pour comparabilité (même fenêtre que 2026)
- Dates du bloc courant portées au 05/10/2026 et 05/10/2025 (B115/D115/K133, L44/N44)
- Rubriques : TOURTEAU SOJA 16 590,9 M / 46 336,9 t ; CONCENTRES 9 881,9 M / 14 748,2 t ; MAIS inchangé (pas de vente en octobre)
- Cohérence Jan-Sep contrôlée : deltas = contribution octobre, tous positifs
- Auteur « William Francis Fohom, Data Analyst » sur les métadonnées du classeur

Co-Authored-By: Claude Code <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/download/ADMINISTRATEUR_DE_VENTE_rempli.xlsx
+++ b/download/ADMINISTRATEUR_DE_VENTE_rempli.xlsx
@@ -3098,11 +3098,11 @@
         </is>
       </c>
       <c r="B115" s="40" t="n">
-        <v>46295</v>
+        <v>46300</v>
       </c>
       <c r="C115" s="41" t="n"/>
       <c r="D115" s="1" t="n">
-        <v>45930</v>
+        <v>45935</v>
       </c>
       <c r="E115" s="2" t="n"/>
       <c r="F115" s="35" t="inlineStr">
@@ -3152,14 +3152,14 @@
         </is>
       </c>
       <c r="B117" s="8" t="n">
-        <v>2896256115.24</v>
+        <v>2947340263.49</v>
       </c>
       <c r="C117" s="9">
         <f>+B117/$B$131</f>
         <v/>
       </c>
       <c r="D117" s="8" t="n">
-        <v>2041232489</v>
+        <v>2094409449</v>
       </c>
       <c r="E117" s="9">
         <f>+D117/D131</f>
@@ -3186,14 +3186,14 @@
         </is>
       </c>
       <c r="B118" s="8" t="n">
-        <v>1677859022.31</v>
+        <v>1702851892.31</v>
       </c>
       <c r="C118" s="9">
         <f>+B118/$B$131</f>
         <v/>
       </c>
       <c r="D118" s="8" t="n">
-        <v>1181614830</v>
+        <v>1198785864</v>
       </c>
       <c r="E118" s="9">
         <f>+D118/D131</f>
@@ -3220,14 +3220,14 @@
         </is>
       </c>
       <c r="B119" s="8" t="n">
-        <v>1005583943.74</v>
+        <v>1030777889.88</v>
       </c>
       <c r="C119" s="9">
         <f>+B119/$B$131</f>
         <v/>
       </c>
       <c r="D119" s="8" t="n">
-        <v>679683768</v>
+        <v>691067812</v>
       </c>
       <c r="E119" s="9">
         <f>+D119/D131</f>
@@ -3254,14 +3254,14 @@
         </is>
       </c>
       <c r="B120" s="8" t="n">
-        <v>577728822.12</v>
+        <v>589090185.3200001</v>
       </c>
       <c r="C120" s="9">
         <f>+B120/$B$131</f>
         <v/>
       </c>
       <c r="D120" s="8" t="n">
-        <v>366105542</v>
+        <v>377436049</v>
       </c>
       <c r="E120" s="9">
         <f>+D120/D131</f>
@@ -3288,14 +3288,14 @@
         </is>
       </c>
       <c r="B121" s="8" t="n">
-        <v>1418610715.37</v>
+        <v>1435812177.5</v>
       </c>
       <c r="C121" s="9">
         <f>+B121/$B$131</f>
         <v/>
       </c>
       <c r="D121" s="8" t="n">
-        <v>1202508955</v>
+        <v>1221127879</v>
       </c>
       <c r="E121" s="9">
         <f>+D121/D131</f>
@@ -3322,14 +3322,14 @@
         </is>
       </c>
       <c r="B122" s="8" t="n">
-        <v>877622839.51</v>
+        <v>882613634.01</v>
       </c>
       <c r="C122" s="9">
         <f>+B122/$B$131</f>
         <v/>
       </c>
       <c r="D122" s="8" t="n">
-        <v>589782613</v>
+        <v>598400454</v>
       </c>
       <c r="E122" s="9">
         <f>+D122/D131</f>
@@ -3356,14 +3356,14 @@
         </is>
       </c>
       <c r="B123" s="8" t="n">
-        <v>7284344571.38</v>
+        <v>7395777432.18</v>
       </c>
       <c r="C123" s="9">
         <f>+B123/$B$131</f>
         <v/>
       </c>
       <c r="D123" s="8" t="n">
-        <v>6649942780</v>
+        <v>6803541755</v>
       </c>
       <c r="E123" s="9">
         <f>+D123/D131</f>
@@ -3390,14 +3390,14 @@
         </is>
       </c>
       <c r="B124" s="8" t="n">
-        <v>2451046150.95</v>
+        <v>2489659948.39</v>
       </c>
       <c r="C124" s="9">
         <f>+B124/$B$131</f>
         <v/>
       </c>
       <c r="D124" s="8" t="n">
-        <v>1499410596</v>
+        <v>1533576726</v>
       </c>
       <c r="E124" s="9">
         <f>+D124/D131</f>
@@ -3424,14 +3424,14 @@
         </is>
       </c>
       <c r="B125" s="8" t="n">
-        <v>1716103866.29</v>
+        <v>1736215381.78</v>
       </c>
       <c r="C125" s="9">
         <f>+B125/$B$131</f>
         <v/>
       </c>
       <c r="D125" s="8" t="n">
-        <v>1035764760</v>
+        <v>1059218260</v>
       </c>
       <c r="E125" s="9">
         <f>+D125/D131</f>
@@ -3458,14 +3458,14 @@
         </is>
       </c>
       <c r="B126" s="8" t="n">
-        <v>1097141014.61</v>
+        <v>1112679685.88</v>
       </c>
       <c r="C126" s="9">
         <f>+B126/$B$131</f>
         <v/>
       </c>
       <c r="D126" s="8" t="n">
-        <v>1042583624</v>
+        <v>1068953668</v>
       </c>
       <c r="E126" s="9">
         <f>+D126/D131</f>
@@ -3492,14 +3492,14 @@
         </is>
       </c>
       <c r="B127" s="8" t="n">
-        <v>915735275.1799999</v>
+        <v>929560093.3</v>
       </c>
       <c r="C127" s="9">
         <f>+B127/$B$131</f>
         <v/>
       </c>
       <c r="D127" s="8" t="n">
-        <v>921048169</v>
+        <v>936498785</v>
       </c>
       <c r="E127" s="9">
         <f>+D127/D131</f>
@@ -3526,14 +3526,14 @@
         </is>
       </c>
       <c r="B128" s="8" t="n">
-        <v>1547925414.79</v>
+        <v>1575446580.61</v>
       </c>
       <c r="C128" s="9">
         <f>+B128/$B$131</f>
         <v/>
       </c>
       <c r="D128" s="8" t="n">
-        <v>1153123492</v>
+        <v>1175618921</v>
       </c>
       <c r="E128" s="9">
         <f>+D128/D131</f>
@@ -3560,14 +3560,14 @@
         </is>
       </c>
       <c r="B129" s="8" t="n">
-        <v>4091635976.22</v>
+        <v>4149086702.27</v>
       </c>
       <c r="C129" s="9">
         <f>+B129/$B$131</f>
         <v/>
       </c>
       <c r="D129" s="8" t="n">
-        <v>4091814437</v>
+        <v>4128357887</v>
       </c>
       <c r="E129" s="9">
         <f>+D129/D131</f>
@@ -3594,14 +3594,14 @@
         </is>
       </c>
       <c r="B130" s="8" t="n">
-        <v>1111978126.89</v>
+        <v>1135364685.9</v>
       </c>
       <c r="C130" s="9">
         <f>+B130/$B$131</f>
         <v/>
       </c>
       <c r="D130" s="8" t="n">
-        <v>730538340</v>
+        <v>744411131</v>
       </c>
       <c r="E130" s="9">
         <f>+D130/D131</f>
@@ -3661,7 +3661,7 @@
         </is>
       </c>
       <c r="K133" s="1" t="n">
-        <v>46295</v>
+        <v>46300</v>
       </c>
       <c r="L133" s="40" t="inlineStr">
         <is>
@@ -5003,11 +5003,11 @@
         </is>
       </c>
       <c r="L44" s="40" t="n">
-        <v>46295</v>
+        <v>46300</v>
       </c>
       <c r="M44" s="41" t="n"/>
       <c r="N44" s="1" t="n">
-        <v>45930</v>
+        <v>45935</v>
       </c>
       <c r="O44" s="2" t="n"/>
       <c r="P44" s="35" t="inlineStr">
@@ -5059,14 +5059,14 @@
         </is>
       </c>
       <c r="L46" s="18" t="n">
-        <v>16310755815</v>
+        <v>16590875607</v>
       </c>
       <c r="M46" s="13">
         <f>+L46/L$56</f>
         <v/>
       </c>
       <c r="N46" s="18" t="n">
-        <v>10604533532</v>
+        <v>10868567718</v>
       </c>
       <c r="O46" s="13">
         <f>+N46/N$56</f>
@@ -5088,14 +5088,14 @@
         </is>
       </c>
       <c r="L47" s="18" t="n">
-        <v>1013902309.6</v>
+        <v>1024226757.82</v>
       </c>
       <c r="M47" s="13">
         <f>+L47/L$56</f>
         <v/>
       </c>
       <c r="N47" s="18" t="n">
-        <v>1077560769</v>
+        <v>1093644059</v>
       </c>
       <c r="O47" s="13">
         <f>+N47/N$56</f>
@@ -5117,14 +5117,14 @@
         </is>
       </c>
       <c r="L48" s="18" t="n">
-        <v>247885100</v>
+        <v>254300800</v>
       </c>
       <c r="M48" s="13">
         <f>+L48/L$56</f>
         <v/>
       </c>
       <c r="N48" s="18" t="n">
-        <v>122803550</v>
+        <v>126068700</v>
       </c>
       <c r="O48" s="13">
         <f>+N48/N$56</f>
@@ -5146,14 +5146,14 @@
         </is>
       </c>
       <c r="L49" s="18" t="n">
-        <v>749341345</v>
+        <v>767066853</v>
       </c>
       <c r="M49" s="13">
         <f>+L49/L$56</f>
         <v/>
       </c>
       <c r="N49" s="18" t="n">
-        <v>486820586</v>
+        <v>496131263</v>
       </c>
       <c r="O49" s="13">
         <f>+N49/N$56</f>
@@ -5175,14 +5175,14 @@
         </is>
       </c>
       <c r="L50" s="18" t="n">
-        <v>9752418729</v>
+        <v>9881939829</v>
       </c>
       <c r="M50" s="13">
         <f>+L50/L$56</f>
         <v/>
       </c>
       <c r="N50" s="18" t="n">
-        <v>9113080068</v>
+        <v>9252396810</v>
       </c>
       <c r="O50" s="13">
         <f>+N50/N$56</f>
@@ -5204,14 +5204,14 @@
         </is>
       </c>
       <c r="L51" s="18" t="n">
-        <v>177855000</v>
+        <v>178386000</v>
       </c>
       <c r="M51" s="13">
         <f>+L51/L$56</f>
         <v/>
       </c>
       <c r="N51" s="18" t="n">
-        <v>133281400</v>
+        <v>134725400</v>
       </c>
       <c r="O51" s="13">
         <f>+N51/N$56</f>
@@ -5233,14 +5233,14 @@
         </is>
       </c>
       <c r="L52" s="18" t="n">
-        <v>28698050</v>
+        <v>28951700</v>
       </c>
       <c r="M52" s="13">
         <f>+L52/L$56</f>
         <v/>
       </c>
       <c r="N52" s="18" t="n">
-        <v>40376400</v>
+        <v>40897200</v>
       </c>
       <c r="O52" s="13">
         <f>+N52/N$56</f>
@@ -5262,14 +5262,14 @@
         </is>
       </c>
       <c r="L53" s="18" t="n">
-        <v>16989956</v>
+        <v>17085956</v>
       </c>
       <c r="M53" s="13">
         <f>+L53/L$56</f>
         <v/>
       </c>
       <c r="N53" s="18" t="n">
-        <v>20633160</v>
+        <v>20803160</v>
       </c>
       <c r="O53" s="13">
         <f>+N53/N$56</f>
@@ -5291,14 +5291,14 @@
         </is>
       </c>
       <c r="L54" s="18" t="n">
-        <v>27906950</v>
+        <v>28834850</v>
       </c>
       <c r="M54" s="13">
         <f>+L54/L$56</f>
         <v/>
       </c>
       <c r="N54" s="18" t="n">
-        <v>851559250</v>
+        <v>865637350</v>
       </c>
       <c r="O54" s="13">
         <f>+N54/N$56</f>
@@ -5817,10 +5817,10 @@
         </is>
       </c>
       <c r="D24" s="25" t="n">
-        <v>45655.28</v>
+        <v>46336.92</v>
       </c>
       <c r="E24" s="24" t="n">
-        <v>30104.05</v>
+        <v>30963.03</v>
       </c>
       <c r="F24" s="32">
         <f>+D24-E24</f>
@@ -5839,10 +5839,10 @@
         </is>
       </c>
       <c r="D25" s="25" t="n">
-        <v>745.87</v>
+        <v>753.35</v>
       </c>
       <c r="E25" s="24" t="n">
-        <v>796.1</v>
+        <v>808.16</v>
       </c>
       <c r="F25" s="32">
         <f>+D25-E25</f>
@@ -5883,10 +5883,10 @@
         </is>
       </c>
       <c r="D27" s="25" t="n">
-        <v>865.79</v>
+        <v>886.66</v>
       </c>
       <c r="E27" s="24" t="n">
-        <v>562.24</v>
+        <v>573.22</v>
       </c>
       <c r="F27" s="32">
         <f>+D27-E27</f>
@@ -5905,10 +5905,10 @@
         </is>
       </c>
       <c r="D28" s="25" t="n">
-        <v>14555.04</v>
+        <v>14748.16</v>
       </c>
       <c r="E28" s="24" t="n">
-        <v>13787.11</v>
+        <v>13999.27</v>
       </c>
       <c r="F28" s="32">
         <f>+D28-E28</f>
@@ -5927,10 +5927,10 @@
         </is>
       </c>
       <c r="D29" s="25" t="n">
-        <v>7.54</v>
+        <v>7.6</v>
       </c>
       <c r="E29" s="24" t="n">
-        <v>11.21</v>
+        <v>11.36</v>
       </c>
       <c r="F29" s="32">
         <f>+D29-E29</f>

</xml_diff>